<commit_message>
updated, feature is finished
</commit_message>
<xml_diff>
--- a/Pemindah JD adaptif V6/TemplateJobDescBaruKosongan/Template GOL 123_Managerial.xlsx
+++ b/Pemindah JD adaptif V6/TemplateJobDescBaruKosongan/Template GOL 123_Managerial.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\titipan Feli\PROYEK GEDE\Database\Template Baru kosong\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\z\TemplateJobDescBaruKosongan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC51C1F-02C5-4A1C-998A-7A3866B87AFF}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F080BBE7-268C-4952-A426-82B5E09CD6B7}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{B4CA32BC-DA9F-4539-8D41-F96D4CBDAEFA}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="56">
   <si>
     <t>JOB DESCRIPTION</t>
   </si>
@@ -165,9 +165,6 @@
     <t>InternalConnection</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>PositionName</t>
   </si>
   <si>
@@ -195,16 +192,10 @@
     <t>Memahami alur proses keseluruhan departemen</t>
   </si>
   <si>
-    <t>1.</t>
-  </si>
-  <si>
     <t>ExternalXYZConnection</t>
   </si>
   <si>
-    <t>2.</t>
-  </si>
-  <si>
-    <t>3.</t>
+    <t>ExternalConnection</t>
   </si>
 </sst>
 </file>
@@ -637,7 +628,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="212">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1137,103 +1128,109 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1715,37 +1712,37 @@
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="5"/>
-      <c r="M2" s="181" t="s">
+      <c r="M2" s="182" t="s">
         <v>0</v>
       </c>
-      <c r="N2" s="182"/>
-      <c r="O2" s="182"/>
-      <c r="P2" s="182"/>
-      <c r="Q2" s="182"/>
-      <c r="R2" s="182"/>
-      <c r="S2" s="182"/>
-      <c r="T2" s="182"/>
-      <c r="U2" s="182"/>
-      <c r="V2" s="182"/>
-      <c r="W2" s="182"/>
-      <c r="X2" s="182"/>
-      <c r="Y2" s="182"/>
-      <c r="Z2" s="182"/>
-      <c r="AA2" s="182"/>
-      <c r="AB2" s="182"/>
-      <c r="AC2" s="182"/>
-      <c r="AD2" s="182"/>
-      <c r="AE2" s="182"/>
-      <c r="AF2" s="182"/>
-      <c r="AG2" s="182"/>
-      <c r="AH2" s="182"/>
-      <c r="AI2" s="182"/>
-      <c r="AJ2" s="182"/>
-      <c r="AK2" s="182"/>
-      <c r="AL2" s="182"/>
-      <c r="AM2" s="182"/>
-      <c r="AN2" s="182"/>
-      <c r="AO2" s="183"/>
+      <c r="N2" s="183"/>
+      <c r="O2" s="183"/>
+      <c r="P2" s="183"/>
+      <c r="Q2" s="183"/>
+      <c r="R2" s="183"/>
+      <c r="S2" s="183"/>
+      <c r="T2" s="183"/>
+      <c r="U2" s="183"/>
+      <c r="V2" s="183"/>
+      <c r="W2" s="183"/>
+      <c r="X2" s="183"/>
+      <c r="Y2" s="183"/>
+      <c r="Z2" s="183"/>
+      <c r="AA2" s="183"/>
+      <c r="AB2" s="183"/>
+      <c r="AC2" s="183"/>
+      <c r="AD2" s="183"/>
+      <c r="AE2" s="183"/>
+      <c r="AF2" s="183"/>
+      <c r="AG2" s="183"/>
+      <c r="AH2" s="183"/>
+      <c r="AI2" s="183"/>
+      <c r="AJ2" s="183"/>
+      <c r="AK2" s="183"/>
+      <c r="AL2" s="183"/>
+      <c r="AM2" s="183"/>
+      <c r="AN2" s="183"/>
+      <c r="AO2" s="184"/>
       <c r="AP2" s="125"/>
       <c r="AQ2" s="126" t="s">
         <v>1</v>
@@ -1779,35 +1776,35 @@
     <row r="3" spans="2:68" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="7"/>
       <c r="L3" s="8"/>
-      <c r="M3" s="184"/>
-      <c r="N3" s="185"/>
-      <c r="O3" s="185"/>
-      <c r="P3" s="185"/>
-      <c r="Q3" s="185"/>
-      <c r="R3" s="185"/>
-      <c r="S3" s="185"/>
-      <c r="T3" s="185"/>
-      <c r="U3" s="185"/>
-      <c r="V3" s="185"/>
-      <c r="W3" s="185"/>
-      <c r="X3" s="185"/>
-      <c r="Y3" s="185"/>
-      <c r="Z3" s="185"/>
-      <c r="AA3" s="185"/>
-      <c r="AB3" s="185"/>
-      <c r="AC3" s="185"/>
-      <c r="AD3" s="185"/>
-      <c r="AE3" s="185"/>
-      <c r="AF3" s="185"/>
-      <c r="AG3" s="185"/>
-      <c r="AH3" s="185"/>
-      <c r="AI3" s="185"/>
-      <c r="AJ3" s="185"/>
-      <c r="AK3" s="185"/>
-      <c r="AL3" s="185"/>
-      <c r="AM3" s="185"/>
-      <c r="AN3" s="185"/>
-      <c r="AO3" s="186"/>
+      <c r="M3" s="185"/>
+      <c r="N3" s="186"/>
+      <c r="O3" s="186"/>
+      <c r="P3" s="186"/>
+      <c r="Q3" s="186"/>
+      <c r="R3" s="186"/>
+      <c r="S3" s="186"/>
+      <c r="T3" s="186"/>
+      <c r="U3" s="186"/>
+      <c r="V3" s="186"/>
+      <c r="W3" s="186"/>
+      <c r="X3" s="186"/>
+      <c r="Y3" s="186"/>
+      <c r="Z3" s="186"/>
+      <c r="AA3" s="186"/>
+      <c r="AB3" s="186"/>
+      <c r="AC3" s="186"/>
+      <c r="AD3" s="186"/>
+      <c r="AE3" s="186"/>
+      <c r="AF3" s="186"/>
+      <c r="AG3" s="186"/>
+      <c r="AH3" s="186"/>
+      <c r="AI3" s="186"/>
+      <c r="AJ3" s="186"/>
+      <c r="AK3" s="186"/>
+      <c r="AL3" s="186"/>
+      <c r="AM3" s="186"/>
+      <c r="AN3" s="186"/>
+      <c r="AO3" s="187"/>
       <c r="AP3" s="129"/>
       <c r="AQ3" s="130"/>
       <c r="AR3" s="130"/>
@@ -1834,35 +1831,35 @@
     <row r="4" spans="2:68" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="7"/>
       <c r="L4" s="8"/>
-      <c r="M4" s="184"/>
-      <c r="N4" s="185"/>
-      <c r="O4" s="185"/>
-      <c r="P4" s="185"/>
-      <c r="Q4" s="185"/>
-      <c r="R4" s="185"/>
-      <c r="S4" s="185"/>
-      <c r="T4" s="185"/>
-      <c r="U4" s="185"/>
-      <c r="V4" s="185"/>
-      <c r="W4" s="185"/>
-      <c r="X4" s="185"/>
-      <c r="Y4" s="185"/>
-      <c r="Z4" s="185"/>
-      <c r="AA4" s="185"/>
-      <c r="AB4" s="185"/>
-      <c r="AC4" s="185"/>
-      <c r="AD4" s="185"/>
-      <c r="AE4" s="185"/>
-      <c r="AF4" s="185"/>
-      <c r="AG4" s="185"/>
-      <c r="AH4" s="185"/>
-      <c r="AI4" s="185"/>
-      <c r="AJ4" s="185"/>
-      <c r="AK4" s="185"/>
-      <c r="AL4" s="185"/>
-      <c r="AM4" s="185"/>
-      <c r="AN4" s="185"/>
-      <c r="AO4" s="186"/>
+      <c r="M4" s="185"/>
+      <c r="N4" s="186"/>
+      <c r="O4" s="186"/>
+      <c r="P4" s="186"/>
+      <c r="Q4" s="186"/>
+      <c r="R4" s="186"/>
+      <c r="S4" s="186"/>
+      <c r="T4" s="186"/>
+      <c r="U4" s="186"/>
+      <c r="V4" s="186"/>
+      <c r="W4" s="186"/>
+      <c r="X4" s="186"/>
+      <c r="Y4" s="186"/>
+      <c r="Z4" s="186"/>
+      <c r="AA4" s="186"/>
+      <c r="AB4" s="186"/>
+      <c r="AC4" s="186"/>
+      <c r="AD4" s="186"/>
+      <c r="AE4" s="186"/>
+      <c r="AF4" s="186"/>
+      <c r="AG4" s="186"/>
+      <c r="AH4" s="186"/>
+      <c r="AI4" s="186"/>
+      <c r="AJ4" s="186"/>
+      <c r="AK4" s="186"/>
+      <c r="AL4" s="186"/>
+      <c r="AM4" s="186"/>
+      <c r="AN4" s="186"/>
+      <c r="AO4" s="187"/>
       <c r="AP4" s="129"/>
       <c r="AQ4" s="130" t="s">
         <v>3</v>
@@ -1905,35 +1902,35 @@
       <c r="J5" s="11"/>
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
-      <c r="M5" s="187"/>
-      <c r="N5" s="188"/>
-      <c r="O5" s="188"/>
-      <c r="P5" s="188"/>
-      <c r="Q5" s="188"/>
-      <c r="R5" s="188"/>
-      <c r="S5" s="188"/>
-      <c r="T5" s="188"/>
-      <c r="U5" s="188"/>
-      <c r="V5" s="188"/>
-      <c r="W5" s="188"/>
-      <c r="X5" s="188"/>
-      <c r="Y5" s="188"/>
-      <c r="Z5" s="188"/>
-      <c r="AA5" s="188"/>
-      <c r="AB5" s="188"/>
-      <c r="AC5" s="188"/>
-      <c r="AD5" s="188"/>
-      <c r="AE5" s="188"/>
-      <c r="AF5" s="188"/>
-      <c r="AG5" s="188"/>
-      <c r="AH5" s="188"/>
-      <c r="AI5" s="188"/>
-      <c r="AJ5" s="188"/>
-      <c r="AK5" s="188"/>
-      <c r="AL5" s="188"/>
-      <c r="AM5" s="188"/>
-      <c r="AN5" s="188"/>
-      <c r="AO5" s="189"/>
+      <c r="M5" s="188"/>
+      <c r="N5" s="189"/>
+      <c r="O5" s="189"/>
+      <c r="P5" s="189"/>
+      <c r="Q5" s="189"/>
+      <c r="R5" s="189"/>
+      <c r="S5" s="189"/>
+      <c r="T5" s="189"/>
+      <c r="U5" s="189"/>
+      <c r="V5" s="189"/>
+      <c r="W5" s="189"/>
+      <c r="X5" s="189"/>
+      <c r="Y5" s="189"/>
+      <c r="Z5" s="189"/>
+      <c r="AA5" s="189"/>
+      <c r="AB5" s="189"/>
+      <c r="AC5" s="189"/>
+      <c r="AD5" s="189"/>
+      <c r="AE5" s="189"/>
+      <c r="AF5" s="189"/>
+      <c r="AG5" s="189"/>
+      <c r="AH5" s="189"/>
+      <c r="AI5" s="189"/>
+      <c r="AJ5" s="189"/>
+      <c r="AK5" s="189"/>
+      <c r="AL5" s="189"/>
+      <c r="AM5" s="189"/>
+      <c r="AN5" s="189"/>
+      <c r="AO5" s="190"/>
       <c r="AP5" s="133"/>
       <c r="AQ5" s="134" t="s">
         <v>4</v>
@@ -2096,99 +2093,99 @@
       <c r="BP7" s="22"/>
     </row>
     <row r="8" spans="2:68" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="178" t="s">
+      <c r="B8" s="193" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="179"/>
-      <c r="D8" s="179"/>
-      <c r="E8" s="179"/>
-      <c r="F8" s="179"/>
-      <c r="G8" s="179"/>
-      <c r="H8" s="179"/>
-      <c r="I8" s="179"/>
-      <c r="J8" s="179"/>
-      <c r="K8" s="179"/>
-      <c r="L8" s="179"/>
-      <c r="M8" s="179"/>
-      <c r="N8" s="179"/>
-      <c r="O8" s="179"/>
-      <c r="P8" s="179"/>
-      <c r="Q8" s="179"/>
-      <c r="R8" s="179"/>
-      <c r="S8" s="179"/>
-      <c r="T8" s="179"/>
-      <c r="U8" s="179"/>
-      <c r="V8" s="179"/>
-      <c r="W8" s="180"/>
-      <c r="X8" s="178" t="s">
+      <c r="C8" s="194"/>
+      <c r="D8" s="194"/>
+      <c r="E8" s="194"/>
+      <c r="F8" s="194"/>
+      <c r="G8" s="194"/>
+      <c r="H8" s="194"/>
+      <c r="I8" s="194"/>
+      <c r="J8" s="194"/>
+      <c r="K8" s="194"/>
+      <c r="L8" s="194"/>
+      <c r="M8" s="194"/>
+      <c r="N8" s="194"/>
+      <c r="O8" s="194"/>
+      <c r="P8" s="194"/>
+      <c r="Q8" s="194"/>
+      <c r="R8" s="194"/>
+      <c r="S8" s="194"/>
+      <c r="T8" s="194"/>
+      <c r="U8" s="194"/>
+      <c r="V8" s="194"/>
+      <c r="W8" s="195"/>
+      <c r="X8" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="Y8" s="179"/>
-      <c r="Z8" s="179"/>
-      <c r="AA8" s="179"/>
-      <c r="AB8" s="179"/>
-      <c r="AC8" s="179"/>
-      <c r="AD8" s="179"/>
-      <c r="AE8" s="179"/>
-      <c r="AF8" s="179"/>
-      <c r="AG8" s="179"/>
-      <c r="AH8" s="179"/>
-      <c r="AI8" s="179"/>
-      <c r="AJ8" s="179"/>
-      <c r="AK8" s="179"/>
-      <c r="AL8" s="179"/>
-      <c r="AM8" s="179"/>
-      <c r="AN8" s="179"/>
-      <c r="AO8" s="180"/>
+      <c r="Y8" s="194"/>
+      <c r="Z8" s="194"/>
+      <c r="AA8" s="194"/>
+      <c r="AB8" s="194"/>
+      <c r="AC8" s="194"/>
+      <c r="AD8" s="194"/>
+      <c r="AE8" s="194"/>
+      <c r="AF8" s="194"/>
+      <c r="AG8" s="194"/>
+      <c r="AH8" s="194"/>
+      <c r="AI8" s="194"/>
+      <c r="AJ8" s="194"/>
+      <c r="AK8" s="194"/>
+      <c r="AL8" s="194"/>
+      <c r="AM8" s="194"/>
+      <c r="AN8" s="194"/>
+      <c r="AO8" s="195"/>
       <c r="AP8" s="24"/>
-      <c r="AQ8" s="178" t="s">
+      <c r="AQ8" s="193" t="s">
         <v>7</v>
       </c>
-      <c r="AR8" s="179"/>
-      <c r="AS8" s="179"/>
-      <c r="AT8" s="179"/>
-      <c r="AU8" s="179"/>
-      <c r="AV8" s="179"/>
-      <c r="AW8" s="179"/>
-      <c r="AX8" s="179"/>
-      <c r="AY8" s="179"/>
-      <c r="AZ8" s="179"/>
-      <c r="BA8" s="179"/>
-      <c r="BB8" s="179"/>
-      <c r="BC8" s="179"/>
-      <c r="BD8" s="179"/>
-      <c r="BE8" s="179"/>
-      <c r="BF8" s="179"/>
-      <c r="BG8" s="179"/>
-      <c r="BH8" s="179"/>
-      <c r="BI8" s="179"/>
-      <c r="BJ8" s="179"/>
-      <c r="BK8" s="180"/>
+      <c r="AR8" s="194"/>
+      <c r="AS8" s="194"/>
+      <c r="AT8" s="194"/>
+      <c r="AU8" s="194"/>
+      <c r="AV8" s="194"/>
+      <c r="AW8" s="194"/>
+      <c r="AX8" s="194"/>
+      <c r="AY8" s="194"/>
+      <c r="AZ8" s="194"/>
+      <c r="BA8" s="194"/>
+      <c r="BB8" s="194"/>
+      <c r="BC8" s="194"/>
+      <c r="BD8" s="194"/>
+      <c r="BE8" s="194"/>
+      <c r="BF8" s="194"/>
+      <c r="BG8" s="194"/>
+      <c r="BH8" s="194"/>
+      <c r="BI8" s="194"/>
+      <c r="BJ8" s="194"/>
+      <c r="BK8" s="195"/>
       <c r="BL8" s="1"/>
       <c r="BN8" s="22"/>
     </row>
     <row r="9" spans="2:68" ht="16.7" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B9" s="7"/>
-      <c r="X9" s="196" t="s">
-        <v>46</v>
-      </c>
-      <c r="Y9" s="197"/>
-      <c r="Z9" s="197"/>
-      <c r="AA9" s="197"/>
-      <c r="AB9" s="197"/>
-      <c r="AC9" s="197"/>
-      <c r="AD9" s="197"/>
-      <c r="AE9" s="197"/>
-      <c r="AF9" s="197"/>
-      <c r="AG9" s="197"/>
-      <c r="AH9" s="197"/>
-      <c r="AI9" s="197"/>
-      <c r="AJ9" s="197"/>
-      <c r="AK9" s="197"/>
-      <c r="AL9" s="197"/>
-      <c r="AM9" s="197"/>
-      <c r="AN9" s="197"/>
-      <c r="AO9" s="198"/>
+      <c r="X9" s="200" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" s="201"/>
+      <c r="Z9" s="201"/>
+      <c r="AA9" s="201"/>
+      <c r="AB9" s="201"/>
+      <c r="AC9" s="201"/>
+      <c r="AD9" s="201"/>
+      <c r="AE9" s="201"/>
+      <c r="AF9" s="201"/>
+      <c r="AG9" s="201"/>
+      <c r="AH9" s="201"/>
+      <c r="AI9" s="201"/>
+      <c r="AJ9" s="201"/>
+      <c r="AK9" s="201"/>
+      <c r="AL9" s="201"/>
+      <c r="AM9" s="201"/>
+      <c r="AN9" s="201"/>
+      <c r="AO9" s="202"/>
       <c r="AP9" s="7"/>
       <c r="AQ9" s="25" t="s">
         <v>8</v>
@@ -2199,24 +2196,24 @@
     </row>
     <row r="10" spans="2:68" ht="16.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="7"/>
-      <c r="X10" s="199"/>
-      <c r="Y10" s="200"/>
-      <c r="Z10" s="200"/>
-      <c r="AA10" s="200"/>
-      <c r="AB10" s="200"/>
-      <c r="AC10" s="200"/>
-      <c r="AD10" s="200"/>
-      <c r="AE10" s="200"/>
-      <c r="AF10" s="200"/>
-      <c r="AG10" s="200"/>
-      <c r="AH10" s="200"/>
-      <c r="AI10" s="200"/>
-      <c r="AJ10" s="200"/>
-      <c r="AK10" s="200"/>
-      <c r="AL10" s="200"/>
-      <c r="AM10" s="200"/>
-      <c r="AN10" s="200"/>
-      <c r="AO10" s="201"/>
+      <c r="X10" s="203"/>
+      <c r="Y10" s="204"/>
+      <c r="Z10" s="204"/>
+      <c r="AA10" s="204"/>
+      <c r="AB10" s="204"/>
+      <c r="AC10" s="204"/>
+      <c r="AD10" s="204"/>
+      <c r="AE10" s="204"/>
+      <c r="AF10" s="204"/>
+      <c r="AG10" s="204"/>
+      <c r="AH10" s="204"/>
+      <c r="AI10" s="204"/>
+      <c r="AJ10" s="204"/>
+      <c r="AK10" s="204"/>
+      <c r="AL10" s="204"/>
+      <c r="AM10" s="204"/>
+      <c r="AN10" s="204"/>
+      <c r="AO10" s="205"/>
       <c r="AP10" s="26"/>
       <c r="AQ10" s="33"/>
       <c r="AR10" s="47"/>
@@ -2240,24 +2237,24 @@
     <row r="11" spans="2:68" ht="16.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="7"/>
       <c r="W11" s="8"/>
-      <c r="X11" s="202"/>
-      <c r="Y11" s="203"/>
-      <c r="Z11" s="203"/>
-      <c r="AA11" s="203"/>
-      <c r="AB11" s="203"/>
-      <c r="AC11" s="203"/>
-      <c r="AD11" s="203"/>
-      <c r="AE11" s="203"/>
-      <c r="AF11" s="203"/>
-      <c r="AG11" s="203"/>
-      <c r="AH11" s="203"/>
-      <c r="AI11" s="203"/>
-      <c r="AJ11" s="203"/>
-      <c r="AK11" s="203"/>
-      <c r="AL11" s="203"/>
-      <c r="AM11" s="203"/>
-      <c r="AN11" s="203"/>
-      <c r="AO11" s="204"/>
+      <c r="X11" s="206"/>
+      <c r="Y11" s="207"/>
+      <c r="Z11" s="207"/>
+      <c r="AA11" s="207"/>
+      <c r="AB11" s="207"/>
+      <c r="AC11" s="207"/>
+      <c r="AD11" s="207"/>
+      <c r="AE11" s="207"/>
+      <c r="AF11" s="207"/>
+      <c r="AG11" s="207"/>
+      <c r="AH11" s="207"/>
+      <c r="AI11" s="207"/>
+      <c r="AJ11" s="207"/>
+      <c r="AK11" s="207"/>
+      <c r="AL11" s="207"/>
+      <c r="AM11" s="207"/>
+      <c r="AN11" s="207"/>
+      <c r="AO11" s="208"/>
       <c r="AP11" s="26"/>
       <c r="AQ11" s="53"/>
       <c r="AR11" s="52"/>
@@ -2282,26 +2279,26 @@
     <row r="12" spans="2:68" ht="16.7" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="7"/>
       <c r="W12" s="8"/>
-      <c r="X12" s="178" t="s">
+      <c r="X12" s="193" t="s">
         <v>9</v>
       </c>
-      <c r="Y12" s="179"/>
-      <c r="Z12" s="179"/>
-      <c r="AA12" s="179"/>
-      <c r="AB12" s="179"/>
-      <c r="AC12" s="179"/>
-      <c r="AD12" s="179"/>
-      <c r="AE12" s="179"/>
-      <c r="AF12" s="179"/>
-      <c r="AG12" s="179"/>
-      <c r="AH12" s="179"/>
-      <c r="AI12" s="179"/>
-      <c r="AJ12" s="179"/>
-      <c r="AK12" s="179"/>
-      <c r="AL12" s="179"/>
-      <c r="AM12" s="179"/>
-      <c r="AN12" s="179"/>
-      <c r="AO12" s="180"/>
+      <c r="Y12" s="194"/>
+      <c r="Z12" s="194"/>
+      <c r="AA12" s="194"/>
+      <c r="AB12" s="194"/>
+      <c r="AC12" s="194"/>
+      <c r="AD12" s="194"/>
+      <c r="AE12" s="194"/>
+      <c r="AF12" s="194"/>
+      <c r="AG12" s="194"/>
+      <c r="AH12" s="194"/>
+      <c r="AI12" s="194"/>
+      <c r="AJ12" s="194"/>
+      <c r="AK12" s="194"/>
+      <c r="AL12" s="194"/>
+      <c r="AM12" s="194"/>
+      <c r="AN12" s="194"/>
+      <c r="AO12" s="195"/>
       <c r="AP12" s="26"/>
       <c r="AQ12" s="112" t="s">
         <v>10</v>
@@ -2677,14 +2674,14 @@
       <c r="K22" s="11"/>
       <c r="L22" s="11"/>
       <c r="M22" s="111" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N22" s="111"/>
       <c r="O22" s="111"/>
       <c r="P22" s="111"/>
       <c r="Q22" s="111"/>
       <c r="R22" s="111" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S22" s="111"/>
       <c r="T22" s="11"/>
@@ -2734,70 +2731,70 @@
       <c r="BN22" s="22"/>
     </row>
     <row r="23" spans="2:68" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="178" t="s">
+      <c r="B23" s="193" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="179"/>
-      <c r="D23" s="179"/>
-      <c r="E23" s="179"/>
-      <c r="F23" s="179"/>
-      <c r="G23" s="179"/>
-      <c r="H23" s="179"/>
-      <c r="I23" s="179"/>
-      <c r="J23" s="179"/>
-      <c r="K23" s="179"/>
-      <c r="L23" s="179"/>
-      <c r="M23" s="179"/>
-      <c r="N23" s="179"/>
-      <c r="O23" s="179"/>
-      <c r="P23" s="179"/>
-      <c r="Q23" s="179"/>
-      <c r="R23" s="179"/>
-      <c r="S23" s="179"/>
-      <c r="T23" s="179"/>
-      <c r="U23" s="179"/>
-      <c r="V23" s="179"/>
-      <c r="W23" s="179"/>
-      <c r="X23" s="179"/>
-      <c r="Y23" s="179"/>
-      <c r="Z23" s="179"/>
-      <c r="AA23" s="179"/>
-      <c r="AB23" s="179"/>
-      <c r="AC23" s="179"/>
-      <c r="AD23" s="179"/>
-      <c r="AE23" s="179"/>
-      <c r="AF23" s="179"/>
-      <c r="AG23" s="179"/>
-      <c r="AH23" s="179"/>
-      <c r="AI23" s="179"/>
-      <c r="AJ23" s="179"/>
-      <c r="AK23" s="179"/>
-      <c r="AL23" s="179"/>
-      <c r="AM23" s="179"/>
-      <c r="AN23" s="179"/>
-      <c r="AO23" s="179"/>
-      <c r="AP23" s="179"/>
-      <c r="AQ23" s="179"/>
-      <c r="AR23" s="179"/>
-      <c r="AS23" s="179"/>
-      <c r="AT23" s="179"/>
-      <c r="AU23" s="179"/>
-      <c r="AV23" s="179"/>
-      <c r="AW23" s="179"/>
-      <c r="AX23" s="179"/>
-      <c r="AY23" s="179"/>
-      <c r="AZ23" s="179"/>
-      <c r="BA23" s="179"/>
-      <c r="BB23" s="179"/>
-      <c r="BC23" s="179"/>
-      <c r="BD23" s="179"/>
-      <c r="BE23" s="179"/>
-      <c r="BF23" s="179"/>
-      <c r="BG23" s="179"/>
-      <c r="BH23" s="179"/>
-      <c r="BI23" s="179"/>
-      <c r="BJ23" s="179"/>
-      <c r="BK23" s="180"/>
+      <c r="C23" s="194"/>
+      <c r="D23" s="194"/>
+      <c r="E23" s="194"/>
+      <c r="F23" s="194"/>
+      <c r="G23" s="194"/>
+      <c r="H23" s="194"/>
+      <c r="I23" s="194"/>
+      <c r="J23" s="194"/>
+      <c r="K23" s="194"/>
+      <c r="L23" s="194"/>
+      <c r="M23" s="194"/>
+      <c r="N23" s="194"/>
+      <c r="O23" s="194"/>
+      <c r="P23" s="194"/>
+      <c r="Q23" s="194"/>
+      <c r="R23" s="194"/>
+      <c r="S23" s="194"/>
+      <c r="T23" s="194"/>
+      <c r="U23" s="194"/>
+      <c r="V23" s="194"/>
+      <c r="W23" s="194"/>
+      <c r="X23" s="194"/>
+      <c r="Y23" s="194"/>
+      <c r="Z23" s="194"/>
+      <c r="AA23" s="194"/>
+      <c r="AB23" s="194"/>
+      <c r="AC23" s="194"/>
+      <c r="AD23" s="194"/>
+      <c r="AE23" s="194"/>
+      <c r="AF23" s="194"/>
+      <c r="AG23" s="194"/>
+      <c r="AH23" s="194"/>
+      <c r="AI23" s="194"/>
+      <c r="AJ23" s="194"/>
+      <c r="AK23" s="194"/>
+      <c r="AL23" s="194"/>
+      <c r="AM23" s="194"/>
+      <c r="AN23" s="194"/>
+      <c r="AO23" s="194"/>
+      <c r="AP23" s="194"/>
+      <c r="AQ23" s="194"/>
+      <c r="AR23" s="194"/>
+      <c r="AS23" s="194"/>
+      <c r="AT23" s="194"/>
+      <c r="AU23" s="194"/>
+      <c r="AV23" s="194"/>
+      <c r="AW23" s="194"/>
+      <c r="AX23" s="194"/>
+      <c r="AY23" s="194"/>
+      <c r="AZ23" s="194"/>
+      <c r="BA23" s="194"/>
+      <c r="BB23" s="194"/>
+      <c r="BC23" s="194"/>
+      <c r="BD23" s="194"/>
+      <c r="BE23" s="194"/>
+      <c r="BF23" s="194"/>
+      <c r="BG23" s="194"/>
+      <c r="BH23" s="194"/>
+      <c r="BI23" s="194"/>
+      <c r="BJ23" s="194"/>
+      <c r="BK23" s="195"/>
     </row>
     <row r="24" spans="2:68" ht="16.7" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B24" s="40" t="s">
@@ -3690,9 +3687,9 @@
       <c r="BK38" s="148"/>
     </row>
     <row r="39" spans="1:68" ht="16.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="208"/>
-      <c r="C39" s="206"/>
-      <c r="D39" s="207"/>
+      <c r="B39" s="180"/>
+      <c r="C39" s="178"/>
+      <c r="D39" s="179"/>
       <c r="E39" s="142"/>
       <c r="F39" s="147"/>
       <c r="G39" s="147"/>
@@ -3730,8 +3727,8 @@
       <c r="AM39" s="142"/>
       <c r="AN39" s="142"/>
       <c r="AO39" s="148"/>
-      <c r="AP39" s="209"/>
-      <c r="AQ39" s="208"/>
+      <c r="AP39" s="181"/>
+      <c r="AQ39" s="180"/>
       <c r="AR39" s="141"/>
       <c r="AS39" s="142"/>
       <c r="AT39" s="142"/>
@@ -3754,75 +3751,75 @@
       <c r="BK39" s="148"/>
     </row>
     <row r="40" spans="1:68" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="205"/>
+      <c r="B40" s="177"/>
       <c r="C40" s="58"/>
       <c r="D40" s="31"/>
       <c r="E40" s="54"/>
     </row>
     <row r="41" spans="1:68" s="1" customFormat="1" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="B41" s="192"/>
-      <c r="C41" s="192"/>
-      <c r="D41" s="192"/>
-      <c r="E41" s="192"/>
-      <c r="F41" s="192"/>
-      <c r="G41" s="192"/>
-      <c r="H41" s="192"/>
-      <c r="I41" s="192"/>
-      <c r="J41" s="192"/>
-      <c r="K41" s="192"/>
-      <c r="L41" s="192"/>
-      <c r="M41" s="192"/>
-      <c r="N41" s="192"/>
-      <c r="O41" s="192"/>
-      <c r="P41" s="192"/>
-      <c r="Q41" s="192"/>
-      <c r="R41" s="192"/>
-      <c r="S41" s="192"/>
-      <c r="T41" s="192"/>
-      <c r="U41" s="192"/>
-      <c r="V41" s="192"/>
-      <c r="W41" s="192"/>
-      <c r="X41" s="192"/>
-      <c r="Y41" s="192"/>
-      <c r="Z41" s="192"/>
-      <c r="AA41" s="192"/>
-      <c r="AB41" s="192"/>
-      <c r="AC41" s="192"/>
-      <c r="AD41" s="192"/>
-      <c r="AE41" s="192"/>
-      <c r="AF41" s="192"/>
-      <c r="AG41" s="192"/>
-      <c r="AH41" s="192"/>
-      <c r="AI41" s="192"/>
-      <c r="AJ41" s="192"/>
-      <c r="AK41" s="192"/>
-      <c r="AL41" s="192"/>
-      <c r="AM41" s="192"/>
-      <c r="AN41" s="192"/>
-      <c r="AO41" s="192"/>
-      <c r="AP41" s="192"/>
-      <c r="AQ41" s="192"/>
-      <c r="AR41" s="192"/>
-      <c r="AS41" s="192"/>
-      <c r="AT41" s="192"/>
-      <c r="AU41" s="192"/>
-      <c r="AV41" s="192"/>
-      <c r="AW41" s="192"/>
-      <c r="AX41" s="192"/>
-      <c r="AY41" s="192"/>
-      <c r="AZ41" s="192"/>
-      <c r="BA41" s="192"/>
-      <c r="BB41" s="192"/>
-      <c r="BC41" s="192"/>
-      <c r="BD41" s="192"/>
-      <c r="BE41" s="192"/>
-      <c r="BF41" s="192"/>
-      <c r="BG41" s="192"/>
-      <c r="BH41" s="192"/>
-      <c r="BI41" s="192"/>
-      <c r="BJ41" s="192"/>
-      <c r="BK41" s="192"/>
+      <c r="B41" s="196"/>
+      <c r="C41" s="196"/>
+      <c r="D41" s="196"/>
+      <c r="E41" s="196"/>
+      <c r="F41" s="196"/>
+      <c r="G41" s="196"/>
+      <c r="H41" s="196"/>
+      <c r="I41" s="196"/>
+      <c r="J41" s="196"/>
+      <c r="K41" s="196"/>
+      <c r="L41" s="196"/>
+      <c r="M41" s="196"/>
+      <c r="N41" s="196"/>
+      <c r="O41" s="196"/>
+      <c r="P41" s="196"/>
+      <c r="Q41" s="196"/>
+      <c r="R41" s="196"/>
+      <c r="S41" s="196"/>
+      <c r="T41" s="196"/>
+      <c r="U41" s="196"/>
+      <c r="V41" s="196"/>
+      <c r="W41" s="196"/>
+      <c r="X41" s="196"/>
+      <c r="Y41" s="196"/>
+      <c r="Z41" s="196"/>
+      <c r="AA41" s="196"/>
+      <c r="AB41" s="196"/>
+      <c r="AC41" s="196"/>
+      <c r="AD41" s="196"/>
+      <c r="AE41" s="196"/>
+      <c r="AF41" s="196"/>
+      <c r="AG41" s="196"/>
+      <c r="AH41" s="196"/>
+      <c r="AI41" s="196"/>
+      <c r="AJ41" s="196"/>
+      <c r="AK41" s="196"/>
+      <c r="AL41" s="196"/>
+      <c r="AM41" s="196"/>
+      <c r="AN41" s="196"/>
+      <c r="AO41" s="196"/>
+      <c r="AP41" s="196"/>
+      <c r="AQ41" s="196"/>
+      <c r="AR41" s="196"/>
+      <c r="AS41" s="196"/>
+      <c r="AT41" s="196"/>
+      <c r="AU41" s="196"/>
+      <c r="AV41" s="196"/>
+      <c r="AW41" s="196"/>
+      <c r="AX41" s="196"/>
+      <c r="AY41" s="196"/>
+      <c r="AZ41" s="196"/>
+      <c r="BA41" s="196"/>
+      <c r="BB41" s="196"/>
+      <c r="BC41" s="196"/>
+      <c r="BD41" s="196"/>
+      <c r="BE41" s="196"/>
+      <c r="BF41" s="196"/>
+      <c r="BG41" s="196"/>
+      <c r="BH41" s="196"/>
+      <c r="BI41" s="196"/>
+      <c r="BJ41" s="196"/>
+      <c r="BK41" s="196"/>
       <c r="BL41" s="2"/>
     </row>
     <row r="42" spans="1:68" ht="21.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
@@ -3837,37 +3834,37 @@
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="5"/>
-      <c r="M42" s="181" t="s">
+      <c r="M42" s="182" t="s">
         <v>0</v>
       </c>
-      <c r="N42" s="182"/>
-      <c r="O42" s="182"/>
-      <c r="P42" s="182"/>
-      <c r="Q42" s="182"/>
-      <c r="R42" s="182"/>
-      <c r="S42" s="182"/>
-      <c r="T42" s="182"/>
-      <c r="U42" s="182"/>
-      <c r="V42" s="182"/>
-      <c r="W42" s="182"/>
-      <c r="X42" s="182"/>
-      <c r="Y42" s="182"/>
-      <c r="Z42" s="182"/>
-      <c r="AA42" s="182"/>
-      <c r="AB42" s="182"/>
-      <c r="AC42" s="182"/>
-      <c r="AD42" s="182"/>
-      <c r="AE42" s="182"/>
-      <c r="AF42" s="182"/>
-      <c r="AG42" s="182"/>
-      <c r="AH42" s="182"/>
-      <c r="AI42" s="182"/>
-      <c r="AJ42" s="182"/>
-      <c r="AK42" s="182"/>
-      <c r="AL42" s="182"/>
-      <c r="AM42" s="182"/>
-      <c r="AN42" s="182"/>
-      <c r="AO42" s="183"/>
+      <c r="N42" s="183"/>
+      <c r="O42" s="183"/>
+      <c r="P42" s="183"/>
+      <c r="Q42" s="183"/>
+      <c r="R42" s="183"/>
+      <c r="S42" s="183"/>
+      <c r="T42" s="183"/>
+      <c r="U42" s="183"/>
+      <c r="V42" s="183"/>
+      <c r="W42" s="183"/>
+      <c r="X42" s="183"/>
+      <c r="Y42" s="183"/>
+      <c r="Z42" s="183"/>
+      <c r="AA42" s="183"/>
+      <c r="AB42" s="183"/>
+      <c r="AC42" s="183"/>
+      <c r="AD42" s="183"/>
+      <c r="AE42" s="183"/>
+      <c r="AF42" s="183"/>
+      <c r="AG42" s="183"/>
+      <c r="AH42" s="183"/>
+      <c r="AI42" s="183"/>
+      <c r="AJ42" s="183"/>
+      <c r="AK42" s="183"/>
+      <c r="AL42" s="183"/>
+      <c r="AM42" s="183"/>
+      <c r="AN42" s="183"/>
+      <c r="AO42" s="184"/>
       <c r="AP42" s="136"/>
       <c r="AQ42" s="126" t="str">
         <f>$AQ$2</f>
@@ -3904,35 +3901,35 @@
     <row r="43" spans="1:68" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="7"/>
       <c r="L43" s="8"/>
-      <c r="M43" s="184"/>
-      <c r="N43" s="185"/>
-      <c r="O43" s="185"/>
-      <c r="P43" s="185"/>
-      <c r="Q43" s="185"/>
-      <c r="R43" s="185"/>
-      <c r="S43" s="185"/>
-      <c r="T43" s="185"/>
-      <c r="U43" s="185"/>
-      <c r="V43" s="185"/>
-      <c r="W43" s="185"/>
-      <c r="X43" s="185"/>
-      <c r="Y43" s="185"/>
-      <c r="Z43" s="185"/>
-      <c r="AA43" s="185"/>
-      <c r="AB43" s="185"/>
-      <c r="AC43" s="185"/>
-      <c r="AD43" s="185"/>
-      <c r="AE43" s="185"/>
-      <c r="AF43" s="185"/>
-      <c r="AG43" s="185"/>
-      <c r="AH43" s="185"/>
-      <c r="AI43" s="185"/>
-      <c r="AJ43" s="185"/>
-      <c r="AK43" s="185"/>
-      <c r="AL43" s="185"/>
-      <c r="AM43" s="185"/>
-      <c r="AN43" s="185"/>
-      <c r="AO43" s="186"/>
+      <c r="M43" s="185"/>
+      <c r="N43" s="186"/>
+      <c r="O43" s="186"/>
+      <c r="P43" s="186"/>
+      <c r="Q43" s="186"/>
+      <c r="R43" s="186"/>
+      <c r="S43" s="186"/>
+      <c r="T43" s="186"/>
+      <c r="U43" s="186"/>
+      <c r="V43" s="186"/>
+      <c r="W43" s="186"/>
+      <c r="X43" s="186"/>
+      <c r="Y43" s="186"/>
+      <c r="Z43" s="186"/>
+      <c r="AA43" s="186"/>
+      <c r="AB43" s="186"/>
+      <c r="AC43" s="186"/>
+      <c r="AD43" s="186"/>
+      <c r="AE43" s="186"/>
+      <c r="AF43" s="186"/>
+      <c r="AG43" s="186"/>
+      <c r="AH43" s="186"/>
+      <c r="AI43" s="186"/>
+      <c r="AJ43" s="186"/>
+      <c r="AK43" s="186"/>
+      <c r="AL43" s="186"/>
+      <c r="AM43" s="186"/>
+      <c r="AN43" s="186"/>
+      <c r="AO43" s="187"/>
       <c r="AP43" s="137"/>
       <c r="AQ43" s="112" t="str">
         <f>$AQ$4</f>
@@ -3968,35 +3965,35 @@
     <row r="44" spans="1:68" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="7"/>
       <c r="L44" s="8"/>
-      <c r="M44" s="184"/>
-      <c r="N44" s="185"/>
-      <c r="O44" s="185"/>
-      <c r="P44" s="185"/>
-      <c r="Q44" s="185"/>
-      <c r="R44" s="185"/>
-      <c r="S44" s="185"/>
-      <c r="T44" s="185"/>
-      <c r="U44" s="185"/>
-      <c r="V44" s="185"/>
-      <c r="W44" s="185"/>
-      <c r="X44" s="185"/>
-      <c r="Y44" s="185"/>
-      <c r="Z44" s="185"/>
-      <c r="AA44" s="185"/>
-      <c r="AB44" s="185"/>
-      <c r="AC44" s="185"/>
-      <c r="AD44" s="185"/>
-      <c r="AE44" s="185"/>
-      <c r="AF44" s="185"/>
-      <c r="AG44" s="185"/>
-      <c r="AH44" s="185"/>
-      <c r="AI44" s="185"/>
-      <c r="AJ44" s="185"/>
-      <c r="AK44" s="185"/>
-      <c r="AL44" s="185"/>
-      <c r="AM44" s="185"/>
-      <c r="AN44" s="185"/>
-      <c r="AO44" s="186"/>
+      <c r="M44" s="185"/>
+      <c r="N44" s="186"/>
+      <c r="O44" s="186"/>
+      <c r="P44" s="186"/>
+      <c r="Q44" s="186"/>
+      <c r="R44" s="186"/>
+      <c r="S44" s="186"/>
+      <c r="T44" s="186"/>
+      <c r="U44" s="186"/>
+      <c r="V44" s="186"/>
+      <c r="W44" s="186"/>
+      <c r="X44" s="186"/>
+      <c r="Y44" s="186"/>
+      <c r="Z44" s="186"/>
+      <c r="AA44" s="186"/>
+      <c r="AB44" s="186"/>
+      <c r="AC44" s="186"/>
+      <c r="AD44" s="186"/>
+      <c r="AE44" s="186"/>
+      <c r="AF44" s="186"/>
+      <c r="AG44" s="186"/>
+      <c r="AH44" s="186"/>
+      <c r="AI44" s="186"/>
+      <c r="AJ44" s="186"/>
+      <c r="AK44" s="186"/>
+      <c r="AL44" s="186"/>
+      <c r="AM44" s="186"/>
+      <c r="AN44" s="186"/>
+      <c r="AO44" s="187"/>
       <c r="AP44" s="138"/>
       <c r="AQ44" s="130"/>
       <c r="AR44" s="130"/>
@@ -4033,35 +4030,35 @@
       <c r="J45" s="11"/>
       <c r="K45" s="11"/>
       <c r="L45" s="12"/>
-      <c r="M45" s="187"/>
-      <c r="N45" s="188"/>
-      <c r="O45" s="188"/>
-      <c r="P45" s="188"/>
-      <c r="Q45" s="188"/>
-      <c r="R45" s="188"/>
-      <c r="S45" s="188"/>
-      <c r="T45" s="188"/>
-      <c r="U45" s="188"/>
-      <c r="V45" s="188"/>
-      <c r="W45" s="188"/>
-      <c r="X45" s="188"/>
-      <c r="Y45" s="188"/>
-      <c r="Z45" s="188"/>
-      <c r="AA45" s="188"/>
-      <c r="AB45" s="188"/>
-      <c r="AC45" s="188"/>
-      <c r="AD45" s="188"/>
-      <c r="AE45" s="188"/>
-      <c r="AF45" s="188"/>
-      <c r="AG45" s="188"/>
-      <c r="AH45" s="188"/>
-      <c r="AI45" s="188"/>
-      <c r="AJ45" s="188"/>
-      <c r="AK45" s="188"/>
-      <c r="AL45" s="188"/>
-      <c r="AM45" s="188"/>
-      <c r="AN45" s="188"/>
-      <c r="AO45" s="189"/>
+      <c r="M45" s="188"/>
+      <c r="N45" s="189"/>
+      <c r="O45" s="189"/>
+      <c r="P45" s="189"/>
+      <c r="Q45" s="189"/>
+      <c r="R45" s="189"/>
+      <c r="S45" s="189"/>
+      <c r="T45" s="189"/>
+      <c r="U45" s="189"/>
+      <c r="V45" s="189"/>
+      <c r="W45" s="189"/>
+      <c r="X45" s="189"/>
+      <c r="Y45" s="189"/>
+      <c r="Z45" s="189"/>
+      <c r="AA45" s="189"/>
+      <c r="AB45" s="189"/>
+      <c r="AC45" s="189"/>
+      <c r="AD45" s="189"/>
+      <c r="AE45" s="189"/>
+      <c r="AF45" s="189"/>
+      <c r="AG45" s="189"/>
+      <c r="AH45" s="189"/>
+      <c r="AI45" s="189"/>
+      <c r="AJ45" s="189"/>
+      <c r="AK45" s="189"/>
+      <c r="AL45" s="189"/>
+      <c r="AM45" s="189"/>
+      <c r="AN45" s="189"/>
+      <c r="AO45" s="190"/>
       <c r="AP45" s="139"/>
       <c r="AQ45" s="134" t="str">
         <f>$AQ$5</f>
@@ -4164,74 +4161,74 @@
       <c r="BP47" s="22"/>
     </row>
     <row r="48" spans="1:68" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="193" t="s">
+      <c r="B48" s="197" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="194"/>
-      <c r="D48" s="194"/>
-      <c r="E48" s="194"/>
-      <c r="F48" s="194"/>
-      <c r="G48" s="194"/>
-      <c r="H48" s="194"/>
-      <c r="I48" s="194"/>
-      <c r="J48" s="194"/>
-      <c r="K48" s="194"/>
-      <c r="L48" s="194"/>
-      <c r="M48" s="194"/>
-      <c r="N48" s="194"/>
-      <c r="O48" s="194"/>
-      <c r="P48" s="194"/>
-      <c r="Q48" s="194"/>
-      <c r="R48" s="194"/>
-      <c r="S48" s="194"/>
-      <c r="T48" s="195"/>
+      <c r="C48" s="198"/>
+      <c r="D48" s="198"/>
+      <c r="E48" s="198"/>
+      <c r="F48" s="198"/>
+      <c r="G48" s="198"/>
+      <c r="H48" s="198"/>
+      <c r="I48" s="198"/>
+      <c r="J48" s="198"/>
+      <c r="K48" s="198"/>
+      <c r="L48" s="198"/>
+      <c r="M48" s="198"/>
+      <c r="N48" s="198"/>
+      <c r="O48" s="198"/>
+      <c r="P48" s="198"/>
+      <c r="Q48" s="198"/>
+      <c r="R48" s="198"/>
+      <c r="S48" s="198"/>
+      <c r="T48" s="199"/>
       <c r="U48" s="1"/>
-      <c r="V48" s="193" t="s">
+      <c r="V48" s="197" t="s">
         <v>17</v>
       </c>
-      <c r="W48" s="194"/>
-      <c r="X48" s="194"/>
-      <c r="Y48" s="194"/>
-      <c r="Z48" s="194"/>
-      <c r="AA48" s="194"/>
-      <c r="AB48" s="194"/>
-      <c r="AC48" s="194"/>
-      <c r="AD48" s="194"/>
-      <c r="AE48" s="194"/>
-      <c r="AF48" s="194"/>
-      <c r="AG48" s="194"/>
-      <c r="AH48" s="194"/>
-      <c r="AI48" s="194"/>
-      <c r="AJ48" s="194"/>
-      <c r="AK48" s="194"/>
-      <c r="AL48" s="194"/>
-      <c r="AM48" s="194"/>
-      <c r="AN48" s="194"/>
-      <c r="AO48" s="195"/>
+      <c r="W48" s="198"/>
+      <c r="X48" s="198"/>
+      <c r="Y48" s="198"/>
+      <c r="Z48" s="198"/>
+      <c r="AA48" s="198"/>
+      <c r="AB48" s="198"/>
+      <c r="AC48" s="198"/>
+      <c r="AD48" s="198"/>
+      <c r="AE48" s="198"/>
+      <c r="AF48" s="198"/>
+      <c r="AG48" s="198"/>
+      <c r="AH48" s="198"/>
+      <c r="AI48" s="198"/>
+      <c r="AJ48" s="198"/>
+      <c r="AK48" s="198"/>
+      <c r="AL48" s="198"/>
+      <c r="AM48" s="198"/>
+      <c r="AN48" s="198"/>
+      <c r="AO48" s="199"/>
       <c r="AP48" s="1"/>
-      <c r="AQ48" s="193" t="s">
+      <c r="AQ48" s="197" t="s">
         <v>18</v>
       </c>
-      <c r="AR48" s="194"/>
-      <c r="AS48" s="194"/>
-      <c r="AT48" s="194"/>
-      <c r="AU48" s="194"/>
-      <c r="AV48" s="194"/>
-      <c r="AW48" s="194"/>
-      <c r="AX48" s="194"/>
-      <c r="AY48" s="194"/>
-      <c r="AZ48" s="194"/>
-      <c r="BA48" s="194"/>
-      <c r="BB48" s="194"/>
-      <c r="BC48" s="194"/>
-      <c r="BD48" s="194"/>
-      <c r="BE48" s="194"/>
-      <c r="BF48" s="194"/>
-      <c r="BG48" s="194"/>
-      <c r="BH48" s="194"/>
-      <c r="BI48" s="194"/>
-      <c r="BJ48" s="194"/>
-      <c r="BK48" s="195"/>
+      <c r="AR48" s="198"/>
+      <c r="AS48" s="198"/>
+      <c r="AT48" s="198"/>
+      <c r="AU48" s="198"/>
+      <c r="AV48" s="198"/>
+      <c r="AW48" s="198"/>
+      <c r="AX48" s="198"/>
+      <c r="AY48" s="198"/>
+      <c r="AZ48" s="198"/>
+      <c r="BA48" s="198"/>
+      <c r="BB48" s="198"/>
+      <c r="BC48" s="198"/>
+      <c r="BD48" s="198"/>
+      <c r="BE48" s="198"/>
+      <c r="BF48" s="198"/>
+      <c r="BG48" s="198"/>
+      <c r="BH48" s="198"/>
+      <c r="BI48" s="198"/>
+      <c r="BJ48" s="198"/>
+      <c r="BK48" s="199"/>
       <c r="BN48" s="22"/>
       <c r="BO48" s="23"/>
       <c r="BP48" s="22"/>
@@ -4279,31 +4276,31 @@
       <c r="BI49" s="55"/>
       <c r="BJ49" s="52"/>
       <c r="BK49" s="68"/>
-      <c r="BO49" s="177"/>
-      <c r="BP49" s="177"/>
-      <c r="BQ49" s="177"/>
-      <c r="BR49" s="177"/>
-      <c r="BS49" s="177"/>
-      <c r="BT49" s="177"/>
-      <c r="BU49" s="177"/>
-      <c r="BV49" s="177"/>
-      <c r="BW49" s="177"/>
-      <c r="BX49" s="177"/>
-      <c r="BY49" s="177"/>
-      <c r="BZ49" s="177"/>
-      <c r="CA49" s="177"/>
-      <c r="CB49" s="177"/>
-      <c r="CC49" s="177"/>
-      <c r="CD49" s="177"/>
-      <c r="CE49" s="177"/>
-      <c r="CF49" s="177"/>
-      <c r="CG49" s="177"/>
-      <c r="CH49" s="177"/>
-      <c r="CI49" s="177"/>
+      <c r="BO49" s="209"/>
+      <c r="BP49" s="209"/>
+      <c r="BQ49" s="209"/>
+      <c r="BR49" s="209"/>
+      <c r="BS49" s="209"/>
+      <c r="BT49" s="209"/>
+      <c r="BU49" s="209"/>
+      <c r="BV49" s="209"/>
+      <c r="BW49" s="209"/>
+      <c r="BX49" s="209"/>
+      <c r="BY49" s="209"/>
+      <c r="BZ49" s="209"/>
+      <c r="CA49" s="209"/>
+      <c r="CB49" s="209"/>
+      <c r="CC49" s="209"/>
+      <c r="CD49" s="209"/>
+      <c r="CE49" s="209"/>
+      <c r="CF49" s="209"/>
+      <c r="CG49" s="209"/>
+      <c r="CH49" s="209"/>
+      <c r="CI49" s="209"/>
     </row>
     <row r="50" spans="2:87" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="160" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C50" s="106"/>
       <c r="D50" s="70"/>
@@ -4676,7 +4673,7 @@
         <v>4</v>
       </c>
       <c r="AR57" s="53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AT57" s="88"/>
       <c r="AU57" s="88"/>
@@ -4821,23 +4818,23 @@
       <c r="BI60" s="88"/>
       <c r="BK60" s="8"/>
       <c r="BO60" s="1"/>
-      <c r="BP60" s="177"/>
-      <c r="BQ60" s="177"/>
-      <c r="BR60" s="177"/>
-      <c r="BS60" s="177"/>
-      <c r="BT60" s="177"/>
-      <c r="BU60" s="177"/>
-      <c r="BV60" s="177"/>
-      <c r="BW60" s="177"/>
-      <c r="BX60" s="177"/>
-      <c r="BY60" s="177"/>
-      <c r="BZ60" s="177"/>
-      <c r="CA60" s="177"/>
-      <c r="CB60" s="177"/>
-      <c r="CC60" s="177"/>
-      <c r="CD60" s="177"/>
-      <c r="CE60" s="177"/>
-      <c r="CF60" s="177"/>
+      <c r="BP60" s="209"/>
+      <c r="BQ60" s="209"/>
+      <c r="BR60" s="209"/>
+      <c r="BS60" s="209"/>
+      <c r="BT60" s="209"/>
+      <c r="BU60" s="209"/>
+      <c r="BV60" s="209"/>
+      <c r="BW60" s="209"/>
+      <c r="BX60" s="209"/>
+      <c r="BY60" s="209"/>
+      <c r="BZ60" s="209"/>
+      <c r="CA60" s="209"/>
+      <c r="CB60" s="209"/>
+      <c r="CC60" s="209"/>
+      <c r="CD60" s="209"/>
+      <c r="CE60" s="209"/>
+      <c r="CF60" s="209"/>
     </row>
     <row r="61" spans="2:87" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="91"/>
@@ -4935,28 +4932,28 @@
       <c r="R63" s="45"/>
       <c r="S63" s="45"/>
       <c r="T63" s="94"/>
-      <c r="V63" s="178" t="s">
+      <c r="V63" s="193" t="s">
         <v>25</v>
       </c>
-      <c r="W63" s="179"/>
-      <c r="X63" s="179"/>
-      <c r="Y63" s="179"/>
-      <c r="Z63" s="179"/>
-      <c r="AA63" s="179"/>
-      <c r="AB63" s="179"/>
-      <c r="AC63" s="179"/>
-      <c r="AD63" s="179"/>
-      <c r="AE63" s="179"/>
-      <c r="AF63" s="179"/>
-      <c r="AG63" s="179"/>
-      <c r="AH63" s="179"/>
-      <c r="AI63" s="179"/>
-      <c r="AJ63" s="179"/>
-      <c r="AK63" s="179"/>
-      <c r="AL63" s="179"/>
-      <c r="AM63" s="179"/>
-      <c r="AN63" s="179"/>
-      <c r="AO63" s="180"/>
+      <c r="W63" s="194"/>
+      <c r="X63" s="194"/>
+      <c r="Y63" s="194"/>
+      <c r="Z63" s="194"/>
+      <c r="AA63" s="194"/>
+      <c r="AB63" s="194"/>
+      <c r="AC63" s="194"/>
+      <c r="AD63" s="194"/>
+      <c r="AE63" s="194"/>
+      <c r="AF63" s="194"/>
+      <c r="AG63" s="194"/>
+      <c r="AH63" s="194"/>
+      <c r="AI63" s="194"/>
+      <c r="AJ63" s="194"/>
+      <c r="AK63" s="194"/>
+      <c r="AL63" s="194"/>
+      <c r="AM63" s="194"/>
+      <c r="AN63" s="194"/>
+      <c r="AO63" s="195"/>
       <c r="AP63" s="37"/>
       <c r="AS63" s="88"/>
       <c r="AT63" s="88"/>
@@ -5311,24 +5308,24 @@
       <c r="AO72" s="8"/>
       <c r="AP72" s="8"/>
       <c r="BK72" s="8"/>
-      <c r="BO72" s="177"/>
-      <c r="BP72" s="177"/>
-      <c r="BQ72" s="177"/>
-      <c r="BR72" s="177"/>
-      <c r="BS72" s="177"/>
-      <c r="BT72" s="177"/>
-      <c r="BU72" s="177"/>
-      <c r="BV72" s="177"/>
-      <c r="BW72" s="177"/>
-      <c r="BX72" s="177"/>
-      <c r="BY72" s="177"/>
-      <c r="BZ72" s="177"/>
-      <c r="CA72" s="177"/>
-      <c r="CB72" s="177"/>
-      <c r="CC72" s="177"/>
-      <c r="CD72" s="177"/>
-      <c r="CE72" s="177"/>
-      <c r="CF72" s="177"/>
+      <c r="BO72" s="209"/>
+      <c r="BP72" s="209"/>
+      <c r="BQ72" s="209"/>
+      <c r="BR72" s="209"/>
+      <c r="BS72" s="209"/>
+      <c r="BT72" s="209"/>
+      <c r="BU72" s="209"/>
+      <c r="BV72" s="209"/>
+      <c r="BW72" s="209"/>
+      <c r="BX72" s="209"/>
+      <c r="BY72" s="209"/>
+      <c r="BZ72" s="209"/>
+      <c r="CA72" s="209"/>
+      <c r="CB72" s="209"/>
+      <c r="CC72" s="209"/>
+      <c r="CD72" s="209"/>
+      <c r="CE72" s="209"/>
+      <c r="CF72" s="209"/>
     </row>
     <row r="73" spans="2:84" x14ac:dyDescent="0.2">
       <c r="B73" s="7"/>
@@ -5373,93 +5370,93 @@
       <c r="BK77" s="12"/>
     </row>
     <row r="78" spans="2:84" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="178" t="s">
+      <c r="B78" s="193" t="s">
         <v>26</v>
       </c>
-      <c r="C78" s="179"/>
-      <c r="D78" s="179"/>
-      <c r="E78" s="179"/>
-      <c r="F78" s="179"/>
-      <c r="G78" s="179"/>
-      <c r="H78" s="179"/>
-      <c r="I78" s="179"/>
-      <c r="J78" s="179"/>
-      <c r="K78" s="179"/>
-      <c r="L78" s="179"/>
-      <c r="M78" s="179"/>
-      <c r="N78" s="179"/>
-      <c r="O78" s="179"/>
-      <c r="P78" s="179"/>
-      <c r="Q78" s="179"/>
-      <c r="R78" s="179"/>
-      <c r="S78" s="179"/>
-      <c r="T78" s="179"/>
-      <c r="U78" s="179"/>
-      <c r="V78" s="179"/>
-      <c r="W78" s="179"/>
-      <c r="X78" s="179"/>
-      <c r="Y78" s="179"/>
-      <c r="Z78" s="179"/>
-      <c r="AA78" s="179"/>
-      <c r="AB78" s="179"/>
-      <c r="AC78" s="179"/>
-      <c r="AD78" s="179"/>
-      <c r="AE78" s="179"/>
-      <c r="AF78" s="179"/>
-      <c r="AG78" s="179"/>
-      <c r="AH78" s="179"/>
-      <c r="AI78" s="179"/>
-      <c r="AJ78" s="179"/>
-      <c r="AK78" s="179"/>
-      <c r="AL78" s="179"/>
-      <c r="AM78" s="179"/>
-      <c r="AN78" s="179"/>
-      <c r="AO78" s="179"/>
-      <c r="AP78" s="179"/>
-      <c r="AQ78" s="179"/>
-      <c r="AR78" s="179"/>
-      <c r="AS78" s="179"/>
-      <c r="AT78" s="179"/>
-      <c r="AU78" s="179"/>
-      <c r="AV78" s="179"/>
-      <c r="AW78" s="179"/>
-      <c r="AX78" s="179"/>
-      <c r="AY78" s="179"/>
-      <c r="AZ78" s="179"/>
-      <c r="BA78" s="179"/>
-      <c r="BB78" s="179"/>
-      <c r="BC78" s="179"/>
-      <c r="BD78" s="179"/>
-      <c r="BE78" s="179"/>
-      <c r="BF78" s="179"/>
-      <c r="BG78" s="179"/>
-      <c r="BH78" s="179"/>
-      <c r="BI78" s="179"/>
-      <c r="BJ78" s="179"/>
-      <c r="BK78" s="180"/>
+      <c r="C78" s="194"/>
+      <c r="D78" s="194"/>
+      <c r="E78" s="194"/>
+      <c r="F78" s="194"/>
+      <c r="G78" s="194"/>
+      <c r="H78" s="194"/>
+      <c r="I78" s="194"/>
+      <c r="J78" s="194"/>
+      <c r="K78" s="194"/>
+      <c r="L78" s="194"/>
+      <c r="M78" s="194"/>
+      <c r="N78" s="194"/>
+      <c r="O78" s="194"/>
+      <c r="P78" s="194"/>
+      <c r="Q78" s="194"/>
+      <c r="R78" s="194"/>
+      <c r="S78" s="194"/>
+      <c r="T78" s="194"/>
+      <c r="U78" s="194"/>
+      <c r="V78" s="194"/>
+      <c r="W78" s="194"/>
+      <c r="X78" s="194"/>
+      <c r="Y78" s="194"/>
+      <c r="Z78" s="194"/>
+      <c r="AA78" s="194"/>
+      <c r="AB78" s="194"/>
+      <c r="AC78" s="194"/>
+      <c r="AD78" s="194"/>
+      <c r="AE78" s="194"/>
+      <c r="AF78" s="194"/>
+      <c r="AG78" s="194"/>
+      <c r="AH78" s="194"/>
+      <c r="AI78" s="194"/>
+      <c r="AJ78" s="194"/>
+      <c r="AK78" s="194"/>
+      <c r="AL78" s="194"/>
+      <c r="AM78" s="194"/>
+      <c r="AN78" s="194"/>
+      <c r="AO78" s="194"/>
+      <c r="AP78" s="194"/>
+      <c r="AQ78" s="194"/>
+      <c r="AR78" s="194"/>
+      <c r="AS78" s="194"/>
+      <c r="AT78" s="194"/>
+      <c r="AU78" s="194"/>
+      <c r="AV78" s="194"/>
+      <c r="AW78" s="194"/>
+      <c r="AX78" s="194"/>
+      <c r="AY78" s="194"/>
+      <c r="AZ78" s="194"/>
+      <c r="BA78" s="194"/>
+      <c r="BB78" s="194"/>
+      <c r="BC78" s="194"/>
+      <c r="BD78" s="194"/>
+      <c r="BE78" s="194"/>
+      <c r="BF78" s="194"/>
+      <c r="BG78" s="194"/>
+      <c r="BH78" s="194"/>
+      <c r="BI78" s="194"/>
+      <c r="BJ78" s="194"/>
+      <c r="BK78" s="195"/>
     </row>
     <row r="79" spans="2:84" ht="13.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="190" t="s">
+      <c r="B79" s="191" t="s">
         <v>27</v>
       </c>
-      <c r="C79" s="191"/>
-      <c r="D79" s="191"/>
-      <c r="E79" s="191"/>
-      <c r="F79" s="191"/>
-      <c r="G79" s="191"/>
-      <c r="H79" s="191"/>
-      <c r="I79" s="191"/>
-      <c r="J79" s="191"/>
-      <c r="K79" s="191"/>
-      <c r="L79" s="191"/>
-      <c r="M79" s="191"/>
-      <c r="N79" s="191"/>
-      <c r="O79" s="191"/>
-      <c r="P79" s="191"/>
-      <c r="Q79" s="191"/>
-      <c r="R79" s="191"/>
-      <c r="S79" s="191"/>
-      <c r="T79" s="191"/>
+      <c r="C79" s="192"/>
+      <c r="D79" s="192"/>
+      <c r="E79" s="192"/>
+      <c r="F79" s="192"/>
+      <c r="G79" s="192"/>
+      <c r="H79" s="192"/>
+      <c r="I79" s="192"/>
+      <c r="J79" s="192"/>
+      <c r="K79" s="192"/>
+      <c r="L79" s="192"/>
+      <c r="M79" s="192"/>
+      <c r="N79" s="192"/>
+      <c r="O79" s="192"/>
+      <c r="P79" s="192"/>
+      <c r="Q79" s="192"/>
+      <c r="R79" s="192"/>
+      <c r="S79" s="192"/>
+      <c r="T79" s="192"/>
       <c r="U79" s="161"/>
       <c r="V79" s="162" t="s">
         <v>28</v>
@@ -5508,7 +5505,7 @@
     </row>
     <row r="80" spans="2:84" x14ac:dyDescent="0.25">
       <c r="B80" s="116" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C80" s="101"/>
       <c r="D80" s="101"/>
@@ -5530,7 +5527,7 @@
       <c r="T80" s="101"/>
       <c r="U80" s="52"/>
       <c r="V80" s="101" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="W80" s="101"/>
       <c r="X80" s="52"/>
@@ -5553,7 +5550,7 @@
       <c r="AO80" s="52"/>
       <c r="AP80" s="52"/>
       <c r="AQ80" s="165" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AR80" s="33"/>
       <c r="AS80" s="52"/>
@@ -5578,7 +5575,7 @@
     </row>
     <row r="81" spans="2:63" x14ac:dyDescent="0.25">
       <c r="B81" s="117" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C81" s="52"/>
       <c r="D81" s="101"/>
@@ -5643,12 +5640,10 @@
       <c r="BK81" s="68"/>
     </row>
     <row r="82" spans="2:63" x14ac:dyDescent="0.25">
-      <c r="B82" s="174" t="s">
-        <v>55</v>
-      </c>
-      <c r="C82" s="33" t="s">
+      <c r="B82" s="210" t="s">
         <v>44</v>
       </c>
+      <c r="C82" s="52"/>
       <c r="D82" s="52"/>
       <c r="E82" s="101"/>
       <c r="F82" s="101"/>
@@ -5667,12 +5662,10 @@
       <c r="S82" s="101"/>
       <c r="T82" s="101"/>
       <c r="U82" s="52"/>
-      <c r="V82" s="118" t="s">
-        <v>55</v>
-      </c>
-      <c r="W82" s="155" t="s">
-        <v>56</v>
-      </c>
+      <c r="V82" s="155" t="s">
+        <v>54</v>
+      </c>
+      <c r="W82" s="52"/>
       <c r="X82" s="52"/>
       <c r="Y82" s="52"/>
       <c r="Z82" s="52"/>
@@ -5692,15 +5685,12 @@
       <c r="AN82" s="52"/>
       <c r="AO82" s="52"/>
       <c r="AP82" s="52"/>
-      <c r="AQ82" s="118" t="s">
+      <c r="AQ82" s="211" t="s">
         <v>55</v>
       </c>
-      <c r="AR82" s="156" t="s">
-        <v>45</v>
-      </c>
+      <c r="AR82" s="156"/>
       <c r="AS82" s="52"/>
       <c r="AT82" s="52"/>
-      <c r="AU82" s="52"/>
       <c r="AV82" s="52"/>
       <c r="AW82" s="52"/>
       <c r="AX82" s="52"/>
@@ -5719,12 +5709,8 @@
       <c r="BK82" s="68"/>
     </row>
     <row r="83" spans="2:63" x14ac:dyDescent="0.25">
-      <c r="B83" s="175" t="s">
-        <v>57</v>
-      </c>
-      <c r="C83" s="33" t="s">
-        <v>45</v>
-      </c>
+      <c r="B83" s="175"/>
+      <c r="C83" s="33"/>
       <c r="D83" s="101"/>
       <c r="E83" s="101"/>
       <c r="F83" s="101"/>
@@ -5743,12 +5729,8 @@
       <c r="S83" s="101"/>
       <c r="T83" s="101"/>
       <c r="U83" s="52"/>
-      <c r="V83" s="118" t="s">
-        <v>57</v>
-      </c>
-      <c r="W83" s="176" t="s">
-        <v>45</v>
-      </c>
+      <c r="V83" s="118"/>
+      <c r="W83" s="176"/>
       <c r="X83" s="52"/>
       <c r="Y83" s="52"/>
       <c r="Z83" s="52"/>
@@ -5768,15 +5750,10 @@
       <c r="AN83" s="52"/>
       <c r="AO83" s="52"/>
       <c r="AP83" s="52"/>
-      <c r="AQ83" s="118" t="s">
-        <v>57</v>
-      </c>
-      <c r="AR83" s="156" t="s">
-        <v>45</v>
-      </c>
+      <c r="AQ83" s="118"/>
+      <c r="AR83" s="156"/>
       <c r="AS83" s="52"/>
       <c r="AT83" s="52"/>
-      <c r="AU83" s="52"/>
       <c r="AV83" s="52"/>
       <c r="AW83" s="52"/>
       <c r="AX83" s="52"/>
@@ -5795,12 +5772,8 @@
       <c r="BK83" s="68"/>
     </row>
     <row r="84" spans="2:63" x14ac:dyDescent="0.25">
-      <c r="B84" s="174" t="s">
-        <v>58</v>
-      </c>
-      <c r="C84" s="157" t="s">
-        <v>45</v>
-      </c>
+      <c r="B84" s="174"/>
+      <c r="C84" s="157"/>
       <c r="D84" s="101"/>
       <c r="E84" s="101"/>
       <c r="F84" s="101"/>
@@ -5819,12 +5792,8 @@
       <c r="S84" s="101"/>
       <c r="T84" s="101"/>
       <c r="U84" s="52"/>
-      <c r="V84" s="102" t="s">
-        <v>58</v>
-      </c>
-      <c r="W84" s="176" t="s">
-        <v>45</v>
-      </c>
+      <c r="V84" s="102"/>
+      <c r="W84" s="176"/>
       <c r="X84" s="52"/>
       <c r="Y84" s="52"/>
       <c r="Z84" s="52"/>
@@ -5844,15 +5813,10 @@
       <c r="AN84" s="52"/>
       <c r="AO84" s="52"/>
       <c r="AP84" s="52"/>
-      <c r="AQ84" s="102" t="s">
-        <v>58</v>
-      </c>
-      <c r="AR84" s="156" t="s">
-        <v>45</v>
-      </c>
+      <c r="AQ84" s="102"/>
+      <c r="AR84" s="156"/>
       <c r="AS84" s="52"/>
       <c r="AT84" s="52"/>
-      <c r="AU84" s="52"/>
       <c r="AV84" s="52"/>
       <c r="AW84" s="52"/>
       <c r="AX84" s="52"/>
@@ -5916,7 +5880,6 @@
       <c r="AR85" s="52"/>
       <c r="AS85" s="52"/>
       <c r="AT85" s="52"/>
-      <c r="AU85" s="52"/>
       <c r="AV85" s="52"/>
       <c r="AW85" s="52"/>
       <c r="AX85" s="52"/>
@@ -5979,8 +5942,6 @@
       <c r="AQ86" s="52"/>
       <c r="AR86" s="52"/>
       <c r="AS86" s="52"/>
-      <c r="AT86" s="52"/>
-      <c r="AU86" s="52"/>
       <c r="AV86" s="52"/>
       <c r="AW86" s="52"/>
       <c r="AX86" s="52"/>
@@ -6182,6 +6143,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="BO49:CI49"/>
+    <mergeCell ref="BP60:CF60"/>
+    <mergeCell ref="V63:AO63"/>
+    <mergeCell ref="BO72:CF72"/>
+    <mergeCell ref="B78:BK78"/>
     <mergeCell ref="M2:AO5"/>
     <mergeCell ref="B79:T79"/>
     <mergeCell ref="B23:BK23"/>
@@ -6195,11 +6161,6 @@
     <mergeCell ref="X8:AO8"/>
     <mergeCell ref="AQ8:BK8"/>
     <mergeCell ref="X9:AO11"/>
-    <mergeCell ref="BO49:CI49"/>
-    <mergeCell ref="BP60:CF60"/>
-    <mergeCell ref="V63:AO63"/>
-    <mergeCell ref="BO72:CF72"/>
-    <mergeCell ref="B78:BK78"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.19685039370078741" bottom="0.19685039370078741" header="3.937007874015748E-2" footer="0.23622047244094491"/>

</xml_diff>